<commit_message>
Add pembelian tracking, kategori & reports
Introduce purchase tracking and product categories. Added PembelianBarang and Supplier models and migration (pembelian_barang) and added kategori enum to data_barang. Enhanced Data_barangController: kategori filtering, supplier list, stricter validation, import error handling, record initial purchases and stock adjustments, tambahStok endpoint. Improved Import_data_barang with validation and kategori cleaning. Updated Data_barang model relation. Revamped Arsip and Laporan logic and many Blade views; added report routes for penjualan_umum, penjualan_member, servis, pembelian. Misc fixes: form routes, modals, DataTables improvements. Run database migrations (php artisan migrate) after pulling.
</commit_message>
<xml_diff>
--- a/public/assets/dist/template/format_data_barang.xlsx
+++ b/public/assets/dist/template/format_data_barang.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nikko\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\pos\public\assets\dist\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7452B2CC-A1A9-4740-8891-C416D1CD6D0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37D596AB-714A-4869-84C8-6FC38BDFF680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7A1893CA-BBC5-4E44-897A-5738778435C0}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Barcode</t>
   </si>
@@ -54,13 +54,19 @@
     <t>Harga Member</t>
   </si>
   <si>
-    <t>Iphone 17 Pro Max</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
     <t>Kucing</t>
+  </si>
+  <si>
+    <t>Kategori</t>
+  </si>
+  <si>
+    <t>vocer</t>
+  </si>
+  <si>
+    <t>Esis</t>
   </si>
 </sst>
 </file>
@@ -439,42 +445,46 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DB08CFB-EACF-4439-8E92-BBB22034A0AD}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -482,41 +492,45 @@
         <v>12345678</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="2">
+        <v>9</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E2" s="2">
+        <v>10</v>
+      </c>
+      <c r="F2" s="2">
         <v>1000</v>
       </c>
-      <c r="F2" s="2">
+      <c r="G2" s="2">
         <v>2000</v>
       </c>
-      <c r="G2" s="2">
+      <c r="H2" s="2">
         <v>1500</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="2">
         <v>123456789</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="2">
+      <c r="C3" s="2"/>
+      <c r="D3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="2">
         <v>10</v>
       </c>
-      <c r="E3" s="2">
+      <c r="F3" s="2">
         <v>90000</v>
       </c>
-      <c r="F3" s="2">
+      <c r="G3" s="2">
         <v>100000</v>
       </c>
-      <c r="G3" s="2">
+      <c r="H3" s="2">
         <v>99000</v>
       </c>
     </row>

</xml_diff>